<commit_message>
scan: seg7 2026-08-12 15:52 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq8_2026-08-12.xlsx
+++ b/output/full_scan/batch_seq8_2026-08-12.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O126"/>
+  <dimension ref="A1:O127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>246.9916985759234</v>
+        <v>246.9916985759233</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>16.8</v>
@@ -5509,21 +5509,21 @@
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>7818</v>
+        <v>7828</v>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>溢泰實業</t>
+          <t>創新服務</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
         <v/>
       </c>
       <c r="D96" s="2" t="n">
-        <v>233.5221599975721</v>
+        <v>235.9480833401725</v>
       </c>
       <c r="E96" s="2" t="n">
-        <v>63.4</v>
+        <v>1760</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -5534,16 +5534,16 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>38.33559222107176</v>
+        <v>51.81498204957301</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>31.83510430186436</v>
+        <v>14.92314083123553</v>
       </c>
       <c r="J96" s="2" t="n">
-        <v>0.6316078875340257</v>
+        <v>1.18689980021755</v>
       </c>
       <c r="K96" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L96" s="2" t="n">
         <v>0</v>
@@ -5552,31 +5552,31 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.1991342808405045</v>
+        <v>21.61284453725857</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>7749</v>
+        <v>7818</v>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>意騰-KY</t>
+          <t>溢泰實業</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>231.422227932162</v>
+        <v>233.5221599975721</v>
       </c>
       <c r="E97" s="2" t="n">
-        <v>359.5</v>
+        <v>63.4</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -5587,13 +5587,13 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>46.33436284633599</v>
+        <v>38.33559222107176</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>29.65766089540883</v>
+        <v>31.83510430186436</v>
       </c>
       <c r="J97" s="2" t="n">
-        <v>0.6658568787234561</v>
+        <v>0.6316078875340257</v>
       </c>
       <c r="K97" s="2" t="n">
         <v>0</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>6.822035749604432</v>
+        <v>-0.1991342808405045</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5615,21 +5615,21 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>7768</v>
+        <v>7749</v>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>頌勝科技</t>
+          <t>意騰-KY</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>229.4868509976092</v>
+        <v>231.422227932162</v>
       </c>
       <c r="E98" s="2" t="n">
-        <v>270</v>
+        <v>359.5</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -5640,13 +5640,13 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>42.04802809881053</v>
+        <v>46.33436284633599</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>44.79458911033825</v>
+        <v>29.65766089540883</v>
       </c>
       <c r="J98" s="2" t="n">
-        <v>1.133211209340853</v>
+        <v>0.6658568787234561</v>
       </c>
       <c r="K98" s="2" t="n">
         <v>0</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>3.510516625562417</v>
+        <v>6.822035749604432</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5668,21 +5668,21 @@
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>7753</v>
+        <v>7768</v>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>星亞</t>
+          <t>頌勝科技</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
         <v/>
       </c>
       <c r="D99" s="2" t="n">
-        <v>223.7254957056748</v>
+        <v>229.4868509976092</v>
       </c>
       <c r="E99" s="2" t="n">
-        <v>37.95</v>
+        <v>270</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -5693,13 +5693,13 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>42.34110352784962</v>
+        <v>42.04802809881053</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>11.81989726853086</v>
+        <v>44.79458911033825</v>
       </c>
       <c r="J99" s="2" t="n">
-        <v>0.6851002352922265</v>
+        <v>1.133211209340853</v>
       </c>
       <c r="K99" s="2" t="n">
         <v>0</v>
@@ -5711,31 +5711,31 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0415413813185479</v>
+        <v>3.510516625562417</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>8024</v>
+        <v>7753</v>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>佑華</t>
+          <t>星亞</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
         <v/>
       </c>
       <c r="D100" s="2" t="n">
-        <v>221.3315784001362</v>
+        <v>223.7254957056748</v>
       </c>
       <c r="E100" s="2" t="n">
-        <v>14</v>
+        <v>37.95</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -5746,16 +5746,16 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>43.84157364936667</v>
+        <v>42.34110352784962</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>16.2041733214541</v>
+        <v>11.81989726853086</v>
       </c>
       <c r="J100" s="2" t="n">
-        <v>0.7813581805301636</v>
+        <v>0.6851002352922265</v>
       </c>
       <c r="K100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L100" s="2" t="n">
         <v>0</v>
@@ -5764,31 +5764,31 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>-0.128965132453518</v>
+        <v>0.0415413813185479</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>macd_golden_cross, market_above_ma60, avoid_chase, hist_turn_positive</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>6894</v>
+        <v>8024</v>
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>衛司特</t>
+          <t>佑華</t>
         </is>
       </c>
       <c r="C101" s="2" t="n">
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>213.3870522239542</v>
+        <v>221.3315784001362</v>
       </c>
       <c r="E101" s="2" t="n">
-        <v>338.5</v>
+        <v>14</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -5799,16 +5799,16 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>49.1488364526429</v>
+        <v>43.84157364936667</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>14.88329600933858</v>
+        <v>16.2041733214541</v>
       </c>
       <c r="J101" s="2" t="n">
-        <v>1.333702871928431</v>
+        <v>0.7813581805301636</v>
       </c>
       <c r="K101" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L101" s="2" t="n">
         <v>0</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>3.255506106825711</v>
+        <v>-0.128965132453518</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5827,21 +5827,21 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>7791</v>
+        <v>6894</v>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>皇家可口</t>
+          <t>衛司特</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
         <v/>
       </c>
       <c r="D102" s="2" t="n">
-        <v>209.4715291093367</v>
+        <v>213.3870522239542</v>
       </c>
       <c r="E102" s="2" t="n">
-        <v>59.2</v>
+        <v>338.5</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -5852,13 +5852,13 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>29.86449025909026</v>
+        <v>49.1488364526429</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>26.4923744694239</v>
+        <v>14.88329600933858</v>
       </c>
       <c r="J102" s="2" t="n">
-        <v>0.8888389229662575</v>
+        <v>1.333702871928431</v>
       </c>
       <c r="K102" s="2" t="n">
         <v>0</v>
@@ -5870,31 +5870,31 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.0715514592375021</v>
+        <v>3.255506106825711</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>6953</v>
+        <v>7791</v>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>家碩</t>
+          <t>皇家可口</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>206.4029936915102</v>
+        <v>209.4715291093367</v>
       </c>
       <c r="E103" s="2" t="n">
-        <v>220</v>
+        <v>59.2</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -5905,16 +5905,16 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>50.68841393336982</v>
+        <v>29.86449025909026</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>8.955039238719444</v>
+        <v>26.4923744694239</v>
       </c>
       <c r="J103" s="2" t="n">
-        <v>0.5204395625562817</v>
+        <v>0.8888389229662575</v>
       </c>
       <c r="K103" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L103" s="2" t="n">
         <v>0</v>
@@ -5923,31 +5923,31 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>2.110362033702977</v>
+        <v>-0.0715514592375021</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>6916</v>
+        <v>6953</v>
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>華凌</t>
+          <t>家碩</t>
         </is>
       </c>
       <c r="C104" s="2" t="n">
         <v/>
       </c>
       <c r="D104" s="2" t="n">
-        <v>196.5361712990588</v>
+        <v>206.4029936915102</v>
       </c>
       <c r="E104" s="2" t="n">
-        <v>18.95</v>
+        <v>220</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -5958,16 +5958,16 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>49.99661786764089</v>
+        <v>50.68841393336982</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>13.55537402965307</v>
+        <v>8.955039238719444</v>
       </c>
       <c r="J104" s="2" t="n">
-        <v>0.3386706340622984</v>
+        <v>0.5204395625562817</v>
       </c>
       <c r="K104" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L104" s="2" t="n">
         <v>0</v>
@@ -5976,31 +5976,31 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.094756304300373</v>
+        <v>2.110362033702977</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>6909</v>
+        <v>6916</v>
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>創控</t>
+          <t>華凌</t>
         </is>
       </c>
       <c r="C105" s="2" t="n">
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>180.0869592144513</v>
+        <v>196.5361712990588</v>
       </c>
       <c r="E105" s="2" t="n">
-        <v>41.9</v>
+        <v>18.95</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -6011,13 +6011,13 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>43.74130804252899</v>
+        <v>49.99661786764089</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>28.09695228244011</v>
+        <v>13.55537402965307</v>
       </c>
       <c r="J105" s="2" t="n">
-        <v>0.6084099844669326</v>
+        <v>0.3386706340622984</v>
       </c>
       <c r="K105" s="2" t="n">
         <v>0</v>
@@ -6029,31 +6029,31 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>0.5127945222542878</v>
+        <v>0.094756304300373</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>7803</v>
+        <v>6909</v>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>雲象科技-創</t>
+          <t>創控</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>178.4394080406096</v>
+        <v>180.0869592144513</v>
       </c>
       <c r="E106" s="2" t="n">
-        <v>19.6</v>
+        <v>41.9</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -6064,13 +6064,13 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>38.08622428044291</v>
+        <v>43.74130804252899</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>21.03727437886049</v>
+        <v>28.09695228244011</v>
       </c>
       <c r="J106" s="2" t="n">
-        <v>0.2638266689922308</v>
+        <v>0.6084099844669326</v>
       </c>
       <c r="K106" s="2" t="n">
         <v>0</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0623039154796933</v>
+        <v>0.5127945222542878</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6092,21 +6092,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>7842</v>
+        <v>7803</v>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>天能綠電</t>
+          <t>雲象科技-創</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
         <v/>
       </c>
       <c r="D107" s="2" t="n">
-        <v>177.9193065075354</v>
+        <v>178.4394080406096</v>
       </c>
       <c r="E107" s="2" t="n">
-        <v>90.5</v>
+        <v>19.6</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -6117,13 +6117,13 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>52.03263658456441</v>
+        <v>38.08622428044291</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>10.75958415539862</v>
+        <v>21.03727437886049</v>
       </c>
       <c r="J107" s="2" t="n">
-        <v>0.8176675689201568</v>
+        <v>0.2638266689922308</v>
       </c>
       <c r="K107" s="2" t="n">
         <v>0</v>
@@ -6135,31 +6135,31 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>2.064603615472225</v>
+        <v>0.0623039154796933</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>7810</v>
+        <v>7842</v>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>捷創科技</t>
+          <t>天能綠電</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
         <v/>
       </c>
       <c r="D108" s="2" t="n">
-        <v>172.7123773626915</v>
+        <v>177.9193065075354</v>
       </c>
       <c r="E108" s="2" t="n">
-        <v>200</v>
+        <v>90.5</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -6170,16 +6170,16 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>54.58227378054248</v>
+        <v>52.03263658456441</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>15.63467593006092</v>
+        <v>10.75958415539862</v>
       </c>
       <c r="J108" s="2" t="n">
-        <v>0.694435237872619</v>
+        <v>0.8176675689201568</v>
       </c>
       <c r="K108" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L108" s="2" t="n">
         <v>0</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>2.296613806497071</v>
+        <v>2.064603615472225</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>6895</v>
+        <v>7810</v>
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>宏碩系統</t>
+          <t>捷創科技</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>170.8879789287524</v>
+        <v>172.7123773626915</v>
       </c>
       <c r="E109" s="2" t="n">
-        <v>117.5</v>
+        <v>200</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -6223,13 +6223,13 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>37.37246211810776</v>
+        <v>54.58227378054248</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>24.48276062517652</v>
+        <v>15.63467593006092</v>
       </c>
       <c r="J109" s="2" t="n">
-        <v>0.4107308084410774</v>
+        <v>0.694435237872619</v>
       </c>
       <c r="K109" s="2" t="n">
         <v>1</v>
@@ -6241,31 +6241,31 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>1.228951179283415</v>
+        <v>2.296613806497071</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, adx_trending</t>
+          <t>market_above_ma60, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>8038</v>
+        <v>6895</v>
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>長園科</t>
+          <t>宏碩系統</t>
         </is>
       </c>
       <c r="C110" s="2" t="n">
         <v/>
       </c>
       <c r="D110" s="2" t="n">
-        <v>163.2139987586051</v>
+        <v>170.8879789287524</v>
       </c>
       <c r="E110" s="2" t="n">
-        <v>32.2</v>
+        <v>117.5</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -6276,16 +6276,16 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>36.59594418042397</v>
+        <v>37.37246211810776</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>20.7521209429352</v>
+        <v>24.48276062517652</v>
       </c>
       <c r="J110" s="2" t="n">
-        <v>0.9942679289071552</v>
+        <v>0.4107308084410774</v>
       </c>
       <c r="K110" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L110" s="2" t="n">
         <v>0</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.107115214807496</v>
+        <v>1.228951179283415</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6304,21 +6304,21 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>6918</v>
+        <v>8038</v>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>愛派司</t>
+          <t>長園科</t>
         </is>
       </c>
       <c r="C111" s="2" t="n">
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>160.8377365371524</v>
+        <v>163.2139987586051</v>
       </c>
       <c r="E111" s="2" t="n">
-        <v>72.8</v>
+        <v>32.2</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -6329,13 +6329,13 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>52.3629500044978</v>
+        <v>36.59594418042397</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>17.34691897124235</v>
+        <v>20.7521209429352</v>
       </c>
       <c r="J111" s="2" t="n">
-        <v>0.4256985325921171</v>
+        <v>0.9942679289071552</v>
       </c>
       <c r="K111" s="2" t="n">
         <v>0</v>
@@ -6347,31 +6347,31 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.2869145503811143</v>
+        <v>0.107115214807496</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, adx_trending</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>6869</v>
+        <v>6918</v>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>雲豹能源</t>
+          <t>愛派司</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>160.0504973698956</v>
+        <v>160.8377365371524</v>
       </c>
       <c r="E112" s="2" t="n">
-        <v>67.3</v>
+        <v>72.8</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -6382,13 +6382,13 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.13250413212772</v>
+        <v>52.3629500044978</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>17.57852961044638</v>
+        <v>17.34691897124235</v>
       </c>
       <c r="J112" s="2" t="n">
-        <v>0.4124401413536953</v>
+        <v>0.4256985325921171</v>
       </c>
       <c r="K112" s="2" t="n">
         <v>0</v>
@@ -6400,31 +6400,31 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.5270080213501043</v>
+        <v>0.2869145503811143</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>6885</v>
+        <v>6869</v>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>全福生技</t>
+          <t>雲豹能源</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
         <v/>
       </c>
       <c r="D113" s="2" t="n">
-        <v>159.0428931133955</v>
+        <v>160.0504973698956</v>
       </c>
       <c r="E113" s="2" t="n">
-        <v>20.5</v>
+        <v>67.3</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -6435,13 +6435,13 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>41.78446462220148</v>
+        <v>44.13250413212772</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>12.33730967896988</v>
+        <v>17.57852961044638</v>
       </c>
       <c r="J113" s="2" t="n">
-        <v>0.9327211721584469</v>
+        <v>0.4124401413536953</v>
       </c>
       <c r="K113" s="2" t="n">
         <v>0</v>
@@ -6453,31 +6453,31 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.0200724888135615</v>
+        <v>0.5270080213501043</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, obv_uptrend</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>7799</v>
+        <v>6885</v>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>禾榮科</t>
+          <t>全福生技</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>156.176215753068</v>
+        <v>159.0428931133955</v>
       </c>
       <c r="E114" s="2" t="n">
-        <v>362</v>
+        <v>20.5</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -6488,13 +6488,13 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>44.71503244161672</v>
+        <v>41.78446462220148</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>19.70270764548374</v>
+        <v>12.33730967896988</v>
       </c>
       <c r="J114" s="2" t="n">
-        <v>0.3605577338185671</v>
+        <v>0.9327211721584469</v>
       </c>
       <c r="K114" s="2" t="n">
         <v>0</v>
@@ -6506,31 +6506,31 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-1.476864125528639</v>
+        <v>0.0200724888135615</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>6997</v>
+        <v>7799</v>
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>博弘</t>
+          <t>禾榮科</t>
         </is>
       </c>
       <c r="C115" s="2" t="n">
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>154.0468515679171</v>
+        <v>156.176215753068</v>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0</v>
+        <v>362</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -6541,13 +6541,13 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>43.11968133409501</v>
+        <v>44.71503244161672</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>11.49307310577802</v>
+        <v>19.70270764548374</v>
       </c>
       <c r="J115" s="2" t="n">
-        <v>0.0055887386915365</v>
+        <v>0.3605577338185671</v>
       </c>
       <c r="K115" s="2" t="n">
         <v>0</v>
@@ -6559,31 +6559,31 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-1.822429259156148</v>
+        <v>-1.476864125528639</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase, liquidity_ok</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>6983</v>
+        <v>6997</v>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>華洋精機</t>
+          <t>博弘</t>
         </is>
       </c>
       <c r="C116" s="2" t="n">
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>143.4235516412223</v>
+        <v>154.0468515679171</v>
       </c>
       <c r="E116" s="2" t="n">
-        <v>297</v>
+        <v>0</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -6594,13 +6594,13 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>37.66661402384938</v>
+        <v>43.11968133409501</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>11.96704827896992</v>
+        <v>11.49307310577802</v>
       </c>
       <c r="J116" s="2" t="n">
-        <v>0.4281868129393021</v>
+        <v>0.0055887386915365</v>
       </c>
       <c r="K116" s="2" t="n">
         <v>0</v>
@@ -6612,31 +6612,31 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.7333763590033442</v>
+        <v>-1.822429259156148</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
+          <t>market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>6928</v>
+        <v>6983</v>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>攸泰科技</t>
+          <t>華洋精機</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
         <v/>
       </c>
       <c r="D117" s="2" t="n">
-        <v>141.661336483884</v>
+        <v>143.4235516412223</v>
       </c>
       <c r="E117" s="2" t="n">
-        <v>48.4</v>
+        <v>297</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -6647,13 +6647,13 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>46.18489241648956</v>
+        <v>37.66661402384938</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>14.42933104731084</v>
+        <v>11.96704827896992</v>
       </c>
       <c r="J117" s="2" t="n">
-        <v>0.1604716711697826</v>
+        <v>0.4281868129393021</v>
       </c>
       <c r="K117" s="2" t="n">
         <v>0</v>
@@ -6665,31 +6665,31 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>-0.2097725405221946</v>
+        <v>0.7333763590033442</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
-          <t>market_above_ma60, avoid_chase</t>
+          <t>ema60_gt_ema120, market_above_ma60, avoid_chase</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>6862</v>
+        <v>6928</v>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>三集瑞-KY</t>
+          <t>攸泰科技</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>141.2165669183745</v>
+        <v>141.661336483884</v>
       </c>
       <c r="E118" s="2" t="n">
-        <v>146</v>
+        <v>48.4</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -6700,13 +6700,13 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>45.40111842107098</v>
+        <v>46.18489241648956</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>19.53814965771956</v>
+        <v>14.42933104731084</v>
       </c>
       <c r="J118" s="2" t="n">
-        <v>0.6733248131129896</v>
+        <v>0.1604716711697826</v>
       </c>
       <c r="K118" s="2" t="n">
         <v>0</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>3.278968965047996</v>
+        <v>-0.2097725405221946</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6728,21 +6728,21 @@
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>7728</v>
+        <v>6862</v>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>光焱科技</t>
+          <t>三集瑞-KY</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
         <v/>
       </c>
       <c r="D119" s="2" t="n">
-        <v>135.3627007859683</v>
+        <v>141.2165669183745</v>
       </c>
       <c r="E119" s="2" t="n">
-        <v>600</v>
+        <v>146</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -6753,16 +6753,16 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>46.04742870771756</v>
+        <v>45.40111842107098</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>17.3089309824384</v>
+        <v>19.53814965771956</v>
       </c>
       <c r="J119" s="2" t="n">
-        <v>0.2819615875945088</v>
+        <v>0.6733248131129896</v>
       </c>
       <c r="K119" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L119" s="2" t="n">
         <v>0</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>5.586158673374989</v>
+        <v>3.278968965047996</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6781,21 +6781,21 @@
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>6925</v>
+        <v>7728</v>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>意藍</t>
+          <t>光焱科技</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>112.9657482471469</v>
+        <v>135.3627007859683</v>
       </c>
       <c r="E120" s="2" t="n">
-        <v>53.8</v>
+        <v>600</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -6806,16 +6806,16 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>44.80632554754253</v>
+        <v>46.04742870771756</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>15.1134817019027</v>
+        <v>17.3089309824384</v>
       </c>
       <c r="J120" s="2" t="n">
-        <v>0.8572288107414855</v>
+        <v>0.2819615875945088</v>
       </c>
       <c r="K120" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L120" s="2" t="n">
         <v>0</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>0.5480944943527462</v>
+        <v>5.586158673374989</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6834,21 +6834,21 @@
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>6873</v>
+        <v>6925</v>
       </c>
       <c r="B121" s="2" t="inlineStr">
         <is>
-          <t>泓德能源</t>
+          <t>意藍</t>
         </is>
       </c>
       <c r="C121" s="2" t="n">
         <v/>
       </c>
       <c r="D121" s="2" t="n">
-        <v>110.6347323608651</v>
+        <v>112.9657482471469</v>
       </c>
       <c r="E121" s="2" t="n">
-        <v>74.90000000000001</v>
+        <v>53.8</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -6859,13 +6859,13 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>35.98704454075934</v>
+        <v>44.80632554754253</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>18.1705102392826</v>
+        <v>15.1134817019027</v>
       </c>
       <c r="J121" s="2" t="n">
-        <v>0.9073236727687046</v>
+        <v>0.8572288107414855</v>
       </c>
       <c r="K121" s="2" t="n">
         <v>0</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.5046415883889697</v>
+        <v>0.5480944943527462</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6887,21 +6887,21 @@
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>7760</v>
+        <v>6873</v>
       </c>
       <c r="B122" s="2" t="inlineStr">
         <is>
-          <t>享溫馨</t>
+          <t>泓德能源</t>
         </is>
       </c>
       <c r="C122" s="2" t="n">
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>106.5854361637308</v>
+        <v>110.6347323608651</v>
       </c>
       <c r="E122" s="2" t="n">
-        <v>32.45</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -6912,13 +6912,13 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>36.07505424544555</v>
+        <v>35.98704454075934</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>13.93898041476421</v>
+        <v>18.1705102392826</v>
       </c>
       <c r="J122" s="2" t="n">
-        <v>0.9141726334355952</v>
+        <v>0.9073236727687046</v>
       </c>
       <c r="K122" s="2" t="n">
         <v>0</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.2078538897215227</v>
+        <v>-0.5046415883889697</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6940,21 +6940,21 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>6971</v>
+        <v>7760</v>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>惠民實業</t>
+          <t>享溫馨</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
         <v/>
       </c>
       <c r="D123" s="2" t="n">
-        <v>68.82277685421251</v>
+        <v>106.5854361637308</v>
       </c>
       <c r="E123" s="2" t="n">
-        <v>25.45</v>
+        <v>32.45</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -6965,13 +6965,13 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>32.02937727740927</v>
+        <v>36.07505424544555</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>18.2581523065624</v>
+        <v>13.93898041476421</v>
       </c>
       <c r="J123" s="2" t="n">
-        <v>0.5487299644971714</v>
+        <v>0.9141726334355952</v>
       </c>
       <c r="K123" s="2" t="n">
         <v>0</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.04753562055993</v>
+        <v>-0.2078538897215227</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -6993,21 +6993,21 @@
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>6934</v>
+        <v>6971</v>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>心誠鎂</t>
+          <t>惠民實業</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
         <v/>
       </c>
       <c r="D124" s="2" t="n">
-        <v>67.07843581119523</v>
+        <v>68.82277685421251</v>
       </c>
       <c r="E124" s="2" t="n">
-        <v>72</v>
+        <v>25.45</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -7018,13 +7018,13 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>43.31133321610401</v>
+        <v>32.02937727740927</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>17.53497758996845</v>
+        <v>18.2581523065624</v>
       </c>
       <c r="J124" s="2" t="n">
-        <v>0.674500131803404</v>
+        <v>0.5487299644971714</v>
       </c>
       <c r="K124" s="2" t="n">
         <v>0</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-0.7236424913295864</v>
+        <v>-0.04753562055993</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7046,21 +7046,21 @@
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>7736</v>
+        <v>6934</v>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>虎山</t>
+          <t>心誠鎂</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
         <v/>
       </c>
       <c r="D125" s="2" t="n">
-        <v>66.2800192058297</v>
+        <v>67.07843581119523</v>
       </c>
       <c r="E125" s="2" t="n">
-        <v>69.90000000000001</v>
+        <v>72</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -7071,13 +7071,13 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>43.10389364274265</v>
+        <v>43.31133321610401</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>16.68658110798352</v>
+        <v>17.53497758996845</v>
       </c>
       <c r="J125" s="2" t="n">
-        <v>0.2363155272004997</v>
+        <v>0.674500131803404</v>
       </c>
       <c r="K125" s="2" t="n">
         <v>0</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.0359104897094267</v>
+        <v>-0.7236424913295864</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7099,52 +7099,105 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
+        <v>7736</v>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>虎山</t>
+        </is>
+      </c>
+      <c r="C126" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D126" s="2" t="n">
+        <v>66.2800192058297</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>69.90000000000001</v>
+      </c>
+      <c r="F126" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G126" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H126" s="2" t="n">
+        <v>43.10389364274265</v>
+      </c>
+      <c r="I126" s="2" t="n">
+        <v>16.68658110798352</v>
+      </c>
+      <c r="J126" s="2" t="n">
+        <v>0.2363155272004997</v>
+      </c>
+      <c r="K126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L126" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M126" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N126" s="2" t="n">
+        <v>0.0359104897094267</v>
+      </c>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>market_above_ma60, avoid_chase</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="n">
         <v>7770</v>
       </c>
-      <c r="B126" s="2" t="inlineStr">
+      <c r="B127" s="2" t="inlineStr">
         <is>
           <t>君曜</t>
         </is>
       </c>
-      <c r="C126" s="2" t="n">
-        <v/>
-      </c>
-      <c r="D126" s="2" t="n">
+      <c r="C127" s="2" t="n">
+        <v/>
+      </c>
+      <c r="D127" s="2" t="n">
         <v>65.26911283244915</v>
       </c>
-      <c r="E126" s="2" t="n">
+      <c r="E127" s="2" t="n">
         <v>39.7</v>
       </c>
-      <c r="F126" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-12</t>
-        </is>
-      </c>
-      <c r="G126" s="2" t="b">
-        <v>0</v>
-      </c>
-      <c r="H126" s="2" t="n">
+      <c r="F127" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+      <c r="G127" s="2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H127" s="2" t="n">
         <v>52.25943458014273</v>
       </c>
-      <c r="I126" s="2" t="n">
+      <c r="I127" s="2" t="n">
         <v>11.83869633559225</v>
       </c>
-      <c r="J126" s="2" t="n">
+      <c r="J127" s="2" t="n">
         <v>0.2012524379421512</v>
       </c>
-      <c r="K126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L126" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M126" s="2" t="n">
-        <v>-1</v>
-      </c>
-      <c r="N126" s="2" t="n">
+      <c r="K127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L127" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M127" s="2" t="n">
+        <v>-1</v>
+      </c>
+      <c r="N127" s="2" t="n">
         <v>1.412702227220152</v>
       </c>
-      <c r="O126" s="2" t="inlineStr">
+      <c r="O127" s="2" t="inlineStr">
         <is>
           <t>market_above_ma60, mfi_strong</t>
         </is>

</xml_diff>